<commit_message>
Add depends_on column and cross-team dependency warnings
- Teams sheet: new depends_on column (col 11) — comma-separated team_keys
  the team depends on (e.g. "func_config")
- generate-report.py / generate-report.js: compute dependency warnings at
  report time — warn if any depended-on team is deferred
- Warning appears in terminal output and as a red band in RELEASE-NOTES.xlsx
  Summary sheet; depends_on cell turns red in Teams sheet if broken
- populate_sprint12.py: interfaces.depends_on = "func_config" (demo data)
- docs/dependency-management-options.md: records all 5 options considered
  with pros/cons and upgrade path notes

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/releases/sprint-12/manifest.xlsx
+++ b/releases/sprint-12/manifest.xlsx
@@ -33,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -65,6 +65,11 @@
         <fgColor rgb="00D9EAD3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE699"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -78,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -87,6 +92,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -542,7 +548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -555,7 +561,8 @@
     <col width="28" customWidth="1" min="8" max="8"/>
     <col width="35" customWidth="1" min="9" max="9"/>
     <col width="25" customWidth="1" min="10" max="10"/>
-    <col width="35" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="35" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -611,6 +618,11 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>depends_on</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>reason_if_deferred</t>
         </is>
       </c>
@@ -663,6 +675,7 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -711,7 +724,12 @@
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>func_config</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -752,7 +770,8 @@
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
         <is>
           <t>ELM-1220 blocked pending sign-off from business deferred to sprint-13</t>
         </is>
@@ -806,6 +825,7 @@
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>